<commit_message>
Actualizacion umbrales datos sisnteticos
Se realiza ajustes a datos sinteticos para recalcular con tercentiles los nuevos umbrales a tener en cuenta para entrenamiento de modelo
</commit_message>
<xml_diff>
--- a/Benchmark_EnergiAI_Teams_72.xlsx
+++ b/Benchmark_EnergiAI_Teams_72.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Estudios Vigentes\ESPECIALIZACION DATA SCIENCE ALURA ORACLE\Hackathon G9 Equipo 72\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Estudios Vigentes\ESPECIALIZACION DATA SCIENCE ALURA ORACLE\Hackathon G9 Equipo 72\Data Science Plan A\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755" tabRatio="857"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7755" tabRatio="857" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="benchmark" sheetId="6" r:id="rId1"/>
+    <sheet name="benchmark Inicial V1" sheetId="6" r:id="rId1"/>
+    <sheet name="benchmark Ajustados V2" sheetId="7" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511" iterateDelta="1E-4"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
   <si>
     <t>Límite de Consumo Vampiro (Fuga Estática)</t>
   </si>
@@ -102,6 +103,42 @@
   </si>
   <si>
     <t>Mayor a 110 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Menor a 8.29 kwh / dia</t>
+  </si>
+  <si>
+    <t>Entre 8.29 y 11.78 kwh / dia</t>
+  </si>
+  <si>
+    <t>Mayor a 11.78 kwh / dia</t>
+  </si>
+  <si>
+    <t>Menor a 3.14 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Entre 3.14 y 5.02 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Mayor a 5.02 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Menor a 19.56 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Entre 19.56 y 27.49 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Mayor a 27.49 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Menor a 27.14 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Entre 27.14 y 38.98 kWh/m²·mes</t>
+  </si>
+  <si>
+    <t>Mayor a 38.98 kWh/m²·mes</t>
   </si>
 </sst>
 </file>
@@ -179,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -194,6 +231,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -497,13 +537,13 @@
       <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
       <c r="I2" s="8"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -513,11 +553,11 @@
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
       <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -527,11 +567,11 @@
       <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -778,4 +818,181 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="52" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="8"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="8"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="9"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="9"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D11" s="9"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="9"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="9"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="9"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="9"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="9"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="9"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="9"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="9"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="9"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>